<commit_message>
update ER dashboard data 2026-07-02 12:30
</commit_message>
<xml_diff>
--- a/docs/reports/daily/ER_Kavach_Unified_KPI_Jul1-Jul1.xlsx
+++ b/docs/reports/daily/ER_Kavach_Unified_KPI_Jul1-Jul1.xlsx
@@ -3026,7 +3026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3046,6 +3046,7 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="46" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3147,6 +3148,11 @@
       </c>
       <c r="Q5" s="15" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="R5" s="15" t="inlineStr">
+        <is>
           <t>Loco Type</t>
         </is>
       </c>
@@ -3224,7 +3230,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q6" s="32" t="inlineStr">
+      <c r="Q6" s="32" t="inlineStr"/>
+      <c r="R6" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3303,7 +3310,8 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-      <c r="Q7" s="32" t="inlineStr">
+      <c r="Q7" s="32" t="inlineStr"/>
+      <c r="R7" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3382,7 +3390,8 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-      <c r="Q8" s="32" t="inlineStr">
+      <c r="Q8" s="32" t="inlineStr"/>
+      <c r="R8" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3461,7 +3470,8 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-      <c r="Q9" s="32" t="inlineStr">
+      <c r="Q9" s="32" t="inlineStr"/>
+      <c r="R9" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3540,7 +3550,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q10" s="32" t="inlineStr">
+      <c r="Q10" s="32" t="inlineStr"/>
+      <c r="R10" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3619,7 +3630,8 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-      <c r="Q11" s="32" t="inlineStr">
+      <c r="Q11" s="32" t="inlineStr"/>
+      <c r="R11" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3698,7 +3710,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q12" s="32" t="inlineStr">
+      <c r="Q12" s="32" t="inlineStr"/>
+      <c r="R12" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3777,7 +3790,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q13" s="32" t="inlineStr">
+      <c r="Q13" s="32" t="inlineStr"/>
+      <c r="R13" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3856,7 +3870,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q14" s="32" t="inlineStr">
+      <c r="Q14" s="32" t="inlineStr"/>
+      <c r="R14" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -3935,7 +3950,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q15" s="32" t="inlineStr">
+      <c r="Q15" s="32" t="inlineStr"/>
+      <c r="R15" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4014,7 +4030,8 @@
           <t>Trip mode</t>
         </is>
       </c>
-      <c r="Q16" s="32" t="inlineStr">
+      <c r="Q16" s="32" t="inlineStr"/>
+      <c r="R16" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4093,7 +4110,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q17" s="32" t="inlineStr">
+      <c r="Q17" s="32" t="inlineStr"/>
+      <c r="R17" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4172,7 +4190,8 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-      <c r="Q18" s="32" t="inlineStr">
+      <c r="Q18" s="32" t="inlineStr"/>
+      <c r="R18" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4251,7 +4270,8 @@
           <t>EB at 0-1 km/h</t>
         </is>
       </c>
-      <c r="Q19" s="32" t="inlineStr">
+      <c r="Q19" s="32" t="inlineStr"/>
+      <c r="R19" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4330,7 +4350,8 @@
           <t>Trip mode</t>
         </is>
       </c>
-      <c r="Q20" s="32" t="inlineStr">
+      <c r="Q20" s="32" t="inlineStr"/>
+      <c r="R20" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4410,7 +4431,8 @@
           <t>Sudden MA drop</t>
         </is>
       </c>
-      <c r="Q21" s="32" t="inlineStr">
+      <c r="Q21" s="32" t="inlineStr"/>
+      <c r="R21" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4489,7 +4511,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q22" s="32" t="inlineStr">
+      <c r="Q22" s="32" t="inlineStr"/>
+      <c r="R22" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4568,7 +4591,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q23" s="32" t="inlineStr">
+      <c r="Q23" s="32" t="inlineStr"/>
+      <c r="R23" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4647,7 +4671,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q24" s="32" t="inlineStr">
+      <c r="Q24" s="32" t="inlineStr"/>
+      <c r="R24" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>
@@ -4726,7 +4751,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q25" s="32" t="inlineStr">
+      <c r="Q25" s="32" t="inlineStr"/>
+      <c r="R25" s="32" t="inlineStr">
         <is>
           <t>HBL</t>
         </is>

</xml_diff>